<commit_message>
Earnings Season Q125 p2
mostly tech earnings and new (basic) defence forecasts
</commit_message>
<xml_diff>
--- a/Financial Analysis/AAPL.xlsx
+++ b/Financial Analysis/AAPL.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28623"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28730"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\antos\Desktop\Financial Analysis\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\antos\Documents\GitHub\FinanceModels\Financial Analysis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2667ACAC-BC48-43A4-8B1D-6C6695039363}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7A1D402B-F206-4351-9656-9E8E5DBF48A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="1" xr2:uid="{9DABBB29-C94C-41BD-A4AD-A53C3313D92F}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{9DABBB29-C94C-41BD-A4AD-A53C3313D92F}"/>
   </bookViews>
   <sheets>
     <sheet name="Main" sheetId="1" r:id="rId1"/>
@@ -911,14 +911,14 @@
         <v>1</v>
       </c>
       <c r="D3" s="12">
-        <v>205.35</v>
+        <v>198.81</v>
       </c>
       <c r="E3" s="2">
-        <v>45781</v>
+        <v>45804</v>
       </c>
       <c r="F3" s="2">
         <f ca="1">TODAY()</f>
-        <v>45781</v>
+        <v>45804</v>
       </c>
       <c r="G3" s="2">
         <v>45861</v>
@@ -942,7 +942,7 @@
       </c>
       <c r="D5" s="3">
         <f>D3*D4</f>
-        <v>3067066.53</v>
+        <v>2969386.398</v>
       </c>
     </row>
     <row r="6" spans="2:7" x14ac:dyDescent="0.3">
@@ -984,7 +984,7 @@
       </c>
       <c r="D9" s="3">
         <f>D5-D8</f>
-        <v>3032330.53</v>
+        <v>2934650.398</v>
       </c>
     </row>
   </sheetData>
@@ -8163,7 +8163,7 @@
       </c>
       <c r="BQ35" s="12">
         <f>Main!D3</f>
-        <v>205.35</v>
+        <v>198.81</v>
       </c>
     </row>
     <row r="36" spans="2:69" x14ac:dyDescent="0.3">
@@ -8173,7 +8173,7 @@
       </c>
       <c r="BQ36" s="11">
         <f>BQ34/BQ35-1</f>
-        <v>-0.16472620891373135</v>
+        <v>-0.13724926814765226</v>
       </c>
     </row>
     <row r="37" spans="2:69" x14ac:dyDescent="0.3">
@@ -10715,13 +10715,13 @@
     <row r="79" spans="2:151" x14ac:dyDescent="0.3">
       <c r="BQ79" s="12">
         <f>Main!D3</f>
-        <v>205.35</v>
+        <v>198.81</v>
       </c>
     </row>
     <row r="80" spans="2:151" x14ac:dyDescent="0.3">
       <c r="BQ80" s="11">
         <f>BQ78/BQ79-1</f>
-        <v>-0.13436628886711866</v>
+        <v>-0.10589063638077978</v>
       </c>
     </row>
   </sheetData>

</xml_diff>